<commit_message>
update sensitivity analysis result
</commit_message>
<xml_diff>
--- a/result/sensitivity.xlsx
+++ b/result/sensitivity.xlsx
@@ -385,16 +385,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>0.07675</v>
+        <v>0.077025</v>
       </c>
       <c r="B2">
-        <v>6.249809659430056E-148</v>
+        <v>2.308728324280074E-147</v>
       </c>
       <c r="C2">
-        <v>0.267125</v>
+        <v>0.2675</v>
       </c>
       <c r="D2">
-        <v>8.221766729351771E-16</v>
+        <v>9.449794499962948E-16</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -402,16 +402,16 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>0.07665</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="B3">
-        <v>5.55361142660021E-148</v>
+        <v>1.43003441619528E-147</v>
       </c>
       <c r="C3">
-        <v>0.268025</v>
+        <v>0.268575</v>
       </c>
       <c r="D3">
-        <v>1.130642950178411E-15</v>
+        <v>1.386967413516723E-15</v>
       </c>
       <c r="E3">
         <v>0.1</v>
@@ -419,16 +419,16 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.07615</v>
+        <v>0.07635</v>
       </c>
       <c r="B4">
-        <v>1.059386735532409E-150</v>
+        <v>3.445256432484319E-150</v>
       </c>
       <c r="C4">
-        <v>0.2692</v>
+        <v>0.269825</v>
       </c>
       <c r="D4">
-        <v>1.693213404095136E-15</v>
+        <v>2.092891136767983E-15</v>
       </c>
       <c r="E4">
         <v>0.2</v>
@@ -436,16 +436,16 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>0.07502499999999999</v>
+        <v>0.07552499999999999</v>
       </c>
       <c r="B5">
-        <v>3.581974376170396E-156</v>
+        <v>1.700258669084898E-154</v>
       </c>
       <c r="C5">
-        <v>0.27035</v>
+        <v>0.27075</v>
       </c>
       <c r="D5">
-        <v>2.440342853915957E-15</v>
+        <v>2.826932371641787E-15</v>
       </c>
       <c r="E5">
         <v>0.3</v>
@@ -453,16 +453,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>0.0738</v>
+        <v>0.0743</v>
       </c>
       <c r="B6">
-        <v>7.847502542005518E-162</v>
+        <v>4.691436570225851E-160</v>
       </c>
       <c r="C6">
-        <v>0.271525</v>
+        <v>0.271875</v>
       </c>
       <c r="D6">
-        <v>3.605119921008042E-15</v>
+        <v>4.05480084907358E-15</v>
       </c>
       <c r="E6">
         <v>0.4</v>
@@ -470,16 +470,16 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>0.0746</v>
+        <v>0.07495</v>
       </c>
       <c r="B7">
-        <v>5.30827671044688E-160</v>
+        <v>7.825772634641915E-159</v>
       </c>
       <c r="C7">
-        <v>0.272775</v>
+        <v>0.27345</v>
       </c>
       <c r="D7">
-        <v>5.397904888690135E-15</v>
+        <v>6.716093145618674E-15</v>
       </c>
       <c r="E7">
         <v>0.5</v>
@@ -487,16 +487,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>0.075625</v>
+        <v>0.075825</v>
       </c>
       <c r="B8">
-        <v>1.049381985754122E-157</v>
+        <v>5.583767284244946E-157</v>
       </c>
       <c r="C8">
-        <v>0.2739</v>
+        <v>0.274475</v>
       </c>
       <c r="D8">
-        <v>7.727104453058648E-15</v>
+        <v>9.522611747400902E-15</v>
       </c>
       <c r="E8">
         <v>0.6000000000000001</v>
@@ -504,16 +504,16 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>0.07665</v>
+        <v>0.076975</v>
       </c>
       <c r="B9">
-        <v>8.441036066665199E-156</v>
+        <v>1.430714086007355E-154</v>
       </c>
       <c r="C9">
-        <v>0.274925</v>
+        <v>0.27535</v>
       </c>
       <c r="D9">
-        <v>1.078996734443251E-14</v>
+        <v>1.248853195388933E-14</v>
       </c>
       <c r="E9">
         <v>0.7000000000000001</v>
@@ -521,16 +521,16 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>0.075725</v>
+        <v>0.0759</v>
       </c>
       <c r="B10">
-        <v>7.456865717537241E-160</v>
+        <v>2.658722704797106E-159</v>
       </c>
       <c r="C10">
-        <v>0.2766</v>
+        <v>0.2773</v>
       </c>
       <c r="D10">
-        <v>1.860622646563359E-14</v>
+        <v>2.349484519658665E-14</v>
       </c>
       <c r="E10">
         <v>0.8</v>
@@ -538,16 +538,16 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>0.049025</v>
+        <v>0.04915</v>
       </c>
       <c r="B11">
-        <v>3.797453602583531E-259</v>
+        <v>1.79987573609023E-258</v>
       </c>
       <c r="C11">
-        <v>0.279475</v>
+        <v>0.27995</v>
       </c>
       <c r="D11">
-        <v>4.902739924768368E-14</v>
+        <v>5.67424216813396E-14</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -555,16 +555,16 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>0.07845000000000001</v>
+        <v>0.0786</v>
       </c>
       <c r="B12">
-        <v>4.70662260370496E-150</v>
+        <v>1.119783724380918E-149</v>
       </c>
       <c r="C12">
-        <v>0.2815</v>
+        <v>0.28215</v>
       </c>
       <c r="D12">
-        <v>9.393530759265901E-14</v>
+        <v>1.158688038363393E-13</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -609,16 +609,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>0.07675</v>
+        <v>0.077025</v>
       </c>
       <c r="B2">
-        <v>6.249809659430056E-148</v>
+        <v>2.308728324280074E-147</v>
       </c>
       <c r="C2">
-        <v>0.267125</v>
+        <v>0.2675</v>
       </c>
       <c r="D2">
-        <v>8.221766729351771E-16</v>
+        <v>9.449794499962948E-16</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -626,16 +626,16 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>0.07675</v>
+        <v>0.076975</v>
       </c>
       <c r="B3">
-        <v>5.327150390198391E-148</v>
+        <v>1.456950073811214E-147</v>
       </c>
       <c r="C3">
-        <v>0.262025</v>
+        <v>0.262975</v>
       </c>
       <c r="D3">
-        <v>1.076284550894675E-16</v>
+        <v>1.584250385966018E-16</v>
       </c>
       <c r="E3">
         <v>0.1</v>
@@ -643,16 +643,16 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.076475</v>
+        <v>0.07667499999999999</v>
       </c>
       <c r="B4">
-        <v>6.807415287402822E-149</v>
+        <v>2.092203102962256E-148</v>
       </c>
       <c r="C4">
-        <v>0.2513</v>
+        <v>0.251975</v>
       </c>
       <c r="D4">
-        <v>1.086878700758105E-18</v>
+        <v>1.469937824319415E-18</v>
       </c>
       <c r="E4">
         <v>0.2</v>
@@ -660,16 +660,16 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>0.076225</v>
+        <v>0.07642500000000001</v>
       </c>
       <c r="B5">
-        <v>1.172319268877532E-149</v>
+        <v>3.021144123815628E-149</v>
       </c>
       <c r="C5">
-        <v>0.235275</v>
+        <v>0.235675</v>
       </c>
       <c r="D5">
-        <v>4.986206315605764E-22</v>
+        <v>6.122809446273696E-22</v>
       </c>
       <c r="E5">
         <v>0.3</v>
@@ -677,16 +677,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>0.076275</v>
+        <v>0.0766</v>
       </c>
       <c r="B6">
-        <v>1.837490935566148E-149</v>
+        <v>1.186526467449125E-148</v>
       </c>
       <c r="C6">
-        <v>0.217075</v>
+        <v>0.2178</v>
       </c>
       <c r="D6">
-        <v>1.333581425764919E-26</v>
+        <v>2.138246723523443E-26</v>
       </c>
       <c r="E6">
         <v>0.4</v>
@@ -694,16 +694,16 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>0.07655000000000001</v>
+        <v>0.076725</v>
       </c>
       <c r="B7">
-        <v>1.271289908841375E-148</v>
+        <v>4.178474797474225E-148</v>
       </c>
       <c r="C7">
-        <v>0.199125</v>
+        <v>0.199675</v>
       </c>
       <c r="D7">
-        <v>3.56491713877177E-32</v>
+        <v>5.499869700338425E-32</v>
       </c>
       <c r="E7">
         <v>0.5</v>
@@ -711,16 +711,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>0.07679999999999999</v>
+        <v>0.077075</v>
       </c>
       <c r="B8">
-        <v>9.860679491164001E-148</v>
+        <v>4.30071186267256E-147</v>
       </c>
       <c r="C8">
-        <v>0.18005</v>
+        <v>0.1808</v>
       </c>
       <c r="D8">
-        <v>1.113934597845441E-39</v>
+        <v>2.389186332877066E-39</v>
       </c>
       <c r="E8">
         <v>0.6000000000000001</v>
@@ -728,16 +728,16 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>0.07704999999999999</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="B9">
-        <v>5.073039892759223E-147</v>
+        <v>1.440132874200981E-146</v>
       </c>
       <c r="C9">
-        <v>0.163925</v>
+        <v>0.1641</v>
       </c>
       <c r="D9">
-        <v>2.122440768396808E-47</v>
+        <v>2.585597671813865E-47</v>
       </c>
       <c r="E9">
         <v>0.7000000000000001</v>
@@ -745,16 +745,16 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>0.0772</v>
+        <v>0.07745</v>
       </c>
       <c r="B10">
-        <v>1.486407314033218E-146</v>
+        <v>3.593933098030856E-146</v>
       </c>
       <c r="C10">
-        <v>0.14715</v>
+        <v>0.14775</v>
       </c>
       <c r="D10">
-        <v>1.965073836285049E-57</v>
+        <v>5.577868153120287E-57</v>
       </c>
       <c r="E10">
         <v>0.8</v>
@@ -762,16 +762,16 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>0.07785</v>
+        <v>0.078125</v>
       </c>
       <c r="B11">
-        <v>6.576771942982111E-145</v>
+        <v>3.063537510289005E-144</v>
       </c>
       <c r="C11">
-        <v>0.1332</v>
+        <v>0.1337</v>
       </c>
       <c r="D11">
-        <v>9.963510126354023E-68</v>
+        <v>2.763304724232375E-67</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -779,16 +779,16 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>0.07875</v>
+        <v>0.078975</v>
       </c>
       <c r="B12">
-        <v>2.511927054311519E-142</v>
+        <v>7.532408706390409E-142</v>
       </c>
       <c r="C12">
-        <v>0.121825</v>
+        <v>0.1222</v>
       </c>
       <c r="D12">
-        <v>4.509843475295553E-78</v>
+        <v>1.146267740045915E-77</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -833,16 +833,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>0.07675</v>
+        <v>0.077025</v>
       </c>
       <c r="B2">
-        <v>6.249809659430056E-148</v>
+        <v>2.308728324280074E-147</v>
       </c>
       <c r="C2">
-        <v>0.267125</v>
+        <v>0.2675</v>
       </c>
       <c r="D2">
-        <v>8.221766729351771E-16</v>
+        <v>9.449794499962948E-16</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -850,16 +850,16 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>0.0767</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="B3">
-        <v>5.009849373567243E-148</v>
+        <v>9.156151833686001E-148</v>
       </c>
       <c r="C3">
-        <v>0.26315</v>
+        <v>0.264075</v>
       </c>
       <c r="D3">
-        <v>1.644334302173976E-16</v>
+        <v>2.390992949721171E-16</v>
       </c>
       <c r="E3">
         <v>0.1</v>
@@ -867,16 +867,16 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.076275</v>
+        <v>0.07645</v>
       </c>
       <c r="B4">
-        <v>9.664152364348379E-151</v>
+        <v>2.518739774140739E-150</v>
       </c>
       <c r="C4">
-        <v>0.253775</v>
+        <v>0.2545</v>
       </c>
       <c r="D4">
-        <v>2.990672519063511E-18</v>
+        <v>4.097971094327076E-18</v>
       </c>
       <c r="E4">
         <v>0.2</v>
@@ -884,16 +884,16 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>0.07552499999999999</v>
+        <v>0.076</v>
       </c>
       <c r="B5">
-        <v>6.148226689886058E-155</v>
+        <v>1.905791816372801E-153</v>
       </c>
       <c r="C5">
-        <v>0.23895</v>
+        <v>0.23925</v>
       </c>
       <c r="D5">
-        <v>2.872836630435873E-21</v>
+        <v>3.297615058889159E-21</v>
       </c>
       <c r="E5">
         <v>0.3</v>
@@ -901,16 +901,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>0.07527499999999999</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="B6">
-        <v>1.133337944778751E-157</v>
+        <v>5.680869439876855E-156</v>
       </c>
       <c r="C6">
-        <v>0.221925</v>
+        <v>0.222575</v>
       </c>
       <c r="D6">
-        <v>2.278909901772505E-25</v>
+        <v>3.317306221142837E-25</v>
       </c>
       <c r="E6">
         <v>0.4</v>
@@ -918,16 +918,16 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>0.077125</v>
+        <v>0.07765</v>
       </c>
       <c r="B7">
-        <v>6.457212406250649E-153</v>
+        <v>1.956310063377217E-151</v>
       </c>
       <c r="C7">
-        <v>0.20505</v>
+        <v>0.205725</v>
       </c>
       <c r="D7">
-        <v>2.300940047474778E-30</v>
+        <v>3.780789123509426E-30</v>
       </c>
       <c r="E7">
         <v>0.5</v>
@@ -935,16 +935,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>0.079275</v>
+        <v>0.079625</v>
       </c>
       <c r="B8">
-        <v>1.01754753986351E-146</v>
+        <v>9.8649705640883E-146</v>
       </c>
       <c r="C8">
-        <v>0.18755</v>
+        <v>0.1883</v>
       </c>
       <c r="D8">
-        <v>9.560531725473252E-37</v>
+        <v>1.965670161880384E-36</v>
       </c>
       <c r="E8">
         <v>0.6000000000000001</v>
@@ -952,16 +952,16 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>0.0815</v>
+        <v>0.082</v>
       </c>
       <c r="B9">
-        <v>1.001066245216265E-141</v>
+        <v>1.519981408619409E-140</v>
       </c>
       <c r="C9">
-        <v>0.171925</v>
+        <v>0.1721</v>
       </c>
       <c r="D9">
-        <v>1.821035536400782E-43</v>
+        <v>2.179095641321725E-43</v>
       </c>
       <c r="E9">
         <v>0.7000000000000001</v>
@@ -969,16 +969,16 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>0.08155</v>
+        <v>0.0818</v>
       </c>
       <c r="B10">
-        <v>1.674356428621017E-142</v>
+        <v>9.118031767158835E-142</v>
       </c>
       <c r="C10">
-        <v>0.156225</v>
+        <v>0.156775</v>
       </c>
       <c r="D10">
-        <v>9.548463948282723E-52</v>
+        <v>2.033874542344825E-51</v>
       </c>
       <c r="E10">
         <v>0.8</v>
@@ -986,16 +986,16 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>0.05205</v>
+        <v>0.05215</v>
       </c>
       <c r="B11">
-        <v>7.687619247725295E-238</v>
+        <v>4.60913016909277E-237</v>
       </c>
       <c r="C11">
-        <v>0.144025</v>
+        <v>0.144325</v>
       </c>
       <c r="D11">
-        <v>2.621684680439435E-59</v>
+        <v>4.37426255931344E-59</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -1003,16 +1003,16 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>0.08497499999999999</v>
+        <v>0.08525000000000001</v>
       </c>
       <c r="B12">
-        <v>5.454072032894635E-133</v>
+        <v>1.908507540945365E-132</v>
       </c>
       <c r="C12">
-        <v>0.13415</v>
+        <v>0.1345</v>
       </c>
       <c r="D12">
-        <v>1.284649567049324E-66</v>
+        <v>2.688686188329272E-66</v>
       </c>
       <c r="E12">
         <v>1</v>

</xml_diff>